<commit_message>
Pierwszy comit, chce zapisać historię
</commit_message>
<xml_diff>
--- a/wyniki_wojcicki_d_gmail_com.xlsx
+++ b/wyniki_wojcicki_d_gmail_com.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -671,10 +671,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>118</t>
-        </is>
+      <c r="A25" t="n">
+        <v>118</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -683,10 +681,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
+      <c r="A26" t="n">
+        <v>56</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -695,10 +691,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>192</t>
-        </is>
+      <c r="A27" t="n">
+        <v>192</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -707,10 +701,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="A28" t="n">
+        <v>14</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -719,10 +711,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="A29" t="n">
+        <v>39</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -731,10 +721,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>146</t>
-        </is>
+      <c r="A30" t="n">
+        <v>146</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -743,10 +731,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
+      <c r="A31" t="n">
+        <v>105</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -755,10 +741,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="A32" t="n">
+        <v>20</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -767,10 +751,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A33" t="n">
+        <v>5</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -779,10 +761,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>182</t>
-        </is>
+      <c r="A34" t="n">
+        <v>182</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -791,10 +771,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A35" t="n">
+        <v>7</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -803,10 +781,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
+      <c r="A36" t="n">
+        <v>104</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -815,10 +791,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
+      <c r="A37" t="n">
+        <v>62</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -827,10 +801,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
+      <c r="A38" t="n">
+        <v>74</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -839,10 +811,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="A39" t="n">
+        <v>29</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -851,10 +821,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="A40" t="n">
+        <v>37</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -863,10 +831,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>139</t>
-        </is>
+      <c r="A41" t="n">
+        <v>139</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -875,10 +841,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>199</t>
-        </is>
+      <c r="A42" t="n">
+        <v>199</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -887,10 +851,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
+      <c r="A43" t="n">
+        <v>84</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -899,14 +861,326 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
+      <c r="A44" t="n">
+        <v>196</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>31</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>79</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>197</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>16</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>141</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>25</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>200</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>14</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>18</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>179</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>111</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>70</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>165</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>130</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>78</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>41</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>131</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>12</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>27</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>45</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>68</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>175</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>133</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>odp_21</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>odp_137</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>odp_5</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>odp_97</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>odp_186</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>odp_57</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>odp_56</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>

</xml_diff>